<commit_message>
Opravene charging session podla starej v.27.3.
</commit_message>
<xml_diff>
--- a/www/ev_charging_sessions.xlsx
+++ b/www/ev_charging_sessions.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H167"/>
+  <dimension ref="A1:K171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -454,6 +454,9 @@
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -497,6 +500,21 @@
           <t>Dovod</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Prebytky (kWh)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Siet (kWh)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Uspora (EUR)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -533,6 +551,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -569,6 +596,15 @@
           <t>test</t>
         </is>
       </c>
+      <c r="I3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -605,6 +641,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -641,6 +686,15 @@
           <t>direct</t>
         </is>
       </c>
+      <c r="I5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -677,6 +731,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -713,6 +776,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -749,6 +821,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -785,6 +866,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -821,6 +911,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -857,6 +956,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -893,6 +1001,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -929,6 +1046,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -965,6 +1091,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1001,6 +1136,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1037,6 +1181,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1073,6 +1226,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1109,6 +1271,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1145,6 +1316,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1181,6 +1361,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1217,6 +1406,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1253,6 +1451,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1289,6 +1496,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1325,6 +1541,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1361,6 +1586,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1397,6 +1631,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1433,6 +1676,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1469,6 +1721,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1505,6 +1766,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1541,6 +1811,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1577,6 +1856,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1613,6 +1901,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1649,6 +1946,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1685,6 +1991,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1721,6 +2036,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1757,6 +2081,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1793,6 +2126,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1829,6 +2171,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1865,6 +2216,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1901,6 +2261,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1937,6 +2306,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1973,6 +2351,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2009,6 +2396,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2045,6 +2441,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2081,6 +2486,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2117,6 +2531,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2153,6 +2576,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2189,6 +2621,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2225,6 +2666,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2261,6 +2711,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2297,6 +2756,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K51" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2333,6 +2801,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K52" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -2369,6 +2846,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K53" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -2405,6 +2891,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -2441,6 +2936,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I55" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K55" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -2477,6 +2981,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -2513,6 +3026,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I57" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K57" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -2549,6 +3071,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I58" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K58" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -2585,6 +3116,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I59" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K59" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -2621,6 +3161,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I60" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J60" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K60" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -2657,6 +3206,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I61" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J61" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K61" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -2693,6 +3251,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I62" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K62" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -2729,6 +3296,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I63" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J63" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K63" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -2765,6 +3341,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I64" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J64" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K64" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -2801,6 +3386,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I65" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J65" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K65" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -2837,6 +3431,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I66" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J66" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K66" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -2873,6 +3476,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I67" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K67" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -2909,6 +3521,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I68" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J68" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K68" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -2945,6 +3566,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I69" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J69" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -2981,6 +3611,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I70" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J70" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K70" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -3017,6 +3656,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I71" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J71" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K71" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -3053,6 +3701,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I72" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J72" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K72" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -3089,6 +3746,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I73" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J73" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K73" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -3125,6 +3791,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I74" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J74" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K74" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -3161,6 +3836,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I75" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J75" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K75" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -3197,6 +3881,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I76" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J76" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K76" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -3233,6 +3926,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I77" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J77" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K77" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -3269,6 +3971,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I78" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J78" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K78" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -3305,6 +4016,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I79" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J79" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K79" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -3341,6 +4061,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I80" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J80" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K80" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -3377,6 +4106,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I81" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J81" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K81" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -3413,6 +4151,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I82" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J82" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K82" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -3449,6 +4196,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I83" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J83" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K83" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -3485,6 +4241,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K84" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -3521,6 +4286,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K85" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -3557,6 +4331,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K86" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -3593,6 +4376,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I87" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J87" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K87" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -3629,6 +4421,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I88" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J88" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K88" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -3665,6 +4466,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K89" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -3701,6 +4511,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I90" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J90" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K90" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -3737,6 +4556,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I91" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J91" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K91" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -3773,6 +4601,15 @@
           <t>ev_disconnected</t>
         </is>
       </c>
+      <c r="I92" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J92" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K92" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -3809,6 +4646,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I93" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J93" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K93" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -3845,6 +4691,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I94" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J94" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K94" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -3881,6 +4736,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I95" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J95" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K95" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -3917,6 +4781,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I96" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J96" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K96" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -3953,6 +4826,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I97" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J97" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K97" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -3989,6 +4871,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I98" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J98" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K98" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -4025,6 +4916,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I99" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J99" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K99" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -4061,6 +4961,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I100" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J100" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K100" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -4097,6 +5006,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I101" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J101" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K101" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -4133,6 +5051,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I102" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J102" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K102" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -4169,6 +5096,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I103" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J103" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K103" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -4205,6 +5141,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I104" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J104" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K104" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -4241,6 +5186,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I105" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J105" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K105" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -4277,6 +5231,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I106" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J106" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K106" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -4313,6 +5276,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I107" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J107" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K107" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -4349,6 +5321,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I108" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J108" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K108" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -4385,6 +5366,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I109" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J109" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K109" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -4421,6 +5411,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I110" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J110" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K110" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -4457,6 +5456,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I111" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J111" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K111" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -4493,6 +5501,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I112" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J112" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K112" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -4529,6 +5546,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I113" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J113" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K113" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -4565,6 +5591,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I114" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J114" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K114" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -4601,6 +5636,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I115" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J115" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K115" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -4637,6 +5681,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I116" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J116" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K116" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -4673,6 +5726,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I117" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J117" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K117" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -4709,6 +5771,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I118" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J118" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K118" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -4745,6 +5816,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I119" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J119" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K119" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -4781,6 +5861,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I120" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J120" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K120" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -4817,6 +5906,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I121" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J121" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K121" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -4853,6 +5951,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I122" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J122" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K122" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -4889,6 +5996,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I123" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J123" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K123" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -4925,6 +6041,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I124" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J124" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K124" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -4961,6 +6086,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I125" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J125" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K125" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -4997,6 +6131,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I126" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J126" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K126" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -5033,6 +6176,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I127" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J127" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K127" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -5069,6 +6221,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I128" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J128" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K128" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -5105,6 +6266,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I129" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J129" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K129" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -5141,6 +6311,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I130" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J130" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K130" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -5177,6 +6356,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I131" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J131" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K131" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -5213,6 +6401,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I132" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J132" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K132" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -5249,6 +6446,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I133" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J133" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K133" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -5285,6 +6491,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I134" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J134" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K134" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -5321,6 +6536,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I135" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J135" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K135" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -5357,6 +6581,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I136" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J136" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K136" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -5393,6 +6626,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I137" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J137" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K137" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -5429,6 +6671,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I138" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J138" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K138" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -5465,6 +6716,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I139" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J139" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K139" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -5501,6 +6761,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I140" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J140" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K140" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -5537,6 +6806,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I141" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J141" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K141" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -5573,6 +6851,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I142" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J142" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K142" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -5609,6 +6896,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I143" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J143" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K143" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -5645,6 +6941,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I144" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J144" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K144" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -5681,6 +6986,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I145" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J145" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K145" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -5717,6 +7031,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I146" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J146" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K146" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -5753,6 +7076,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I147" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J147" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K147" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -5789,6 +7121,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I148" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J148" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K148" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -5825,6 +7166,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I149" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J149" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K149" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -5861,6 +7211,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I150" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J150" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K150" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -5897,6 +7256,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I151" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J151" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K151" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -5933,6 +7301,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I152" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J152" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K152" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -5969,6 +7346,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I153" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J153" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K153" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -6005,6 +7391,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I154" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J154" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K154" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -6041,6 +7436,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I155" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J155" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K155" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -6077,6 +7481,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I156" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J156" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K156" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -6113,6 +7526,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I157" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J157" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K157" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -6149,6 +7571,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I158" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J158" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K158" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -6185,6 +7616,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I159" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J159" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K159" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -6221,6 +7661,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I160" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J160" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K160" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -6257,6 +7706,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I161" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J161" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K161" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -6293,6 +7751,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I162" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J162" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K162" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -6329,6 +7796,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I163" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J163" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K163" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -6365,6 +7841,15 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I164" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J164" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K164" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -6401,6 +7886,15 @@
           <t>completed</t>
         </is>
       </c>
+      <c r="I165" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J165" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K165" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -6437,21 +7931,219 @@
           <t>manual</t>
         </is>
       </c>
+      <c r="I166" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J166" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K166" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="167">
-      <c r="C167" s="4" t="inlineStr">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>22:40</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>mysan</t>
+        </is>
+      </c>
+      <c r="D167" s="3" t="n">
+        <v>0.852</v>
+      </c>
+      <c r="E167" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F167" s="2" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="G167" s="2" t="n">
+        <v>92.90000000000001</v>
+      </c>
+      <c r="H167" s="2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="I167" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J167" s="3" t="n">
+        <v>21.171</v>
+      </c>
+      <c r="K167" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>22:40</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>mysan</t>
+        </is>
+      </c>
+      <c r="D168" s="3" t="n">
+        <v>1.172</v>
+      </c>
+      <c r="E168" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F168" s="2" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="G168" s="2" t="n">
+        <v>95.8</v>
+      </c>
+      <c r="H168" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="I168" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J168" s="3" t="n">
+        <v>21.491</v>
+      </c>
+      <c r="K168" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>00:18</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>mysan</t>
+        </is>
+      </c>
+      <c r="D169" s="3" t="n">
+        <v>0.739</v>
+      </c>
+      <c r="E169" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F169" s="2" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="G169" s="2" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="H169" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="I169" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J169" s="3" t="n">
+        <v>0.739</v>
+      </c>
+      <c r="K169" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>00:56</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>mysan</t>
+        </is>
+      </c>
+      <c r="D170" s="3" t="n">
+        <v>0.157</v>
+      </c>
+      <c r="E170" s="3" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="F170" s="2" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="G170" s="2" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H170" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="I170" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J170" s="3" t="n">
+        <v>0.157</v>
+      </c>
+      <c r="K170" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="C171" s="4" t="inlineStr">
         <is>
           <t>SPOLU:</t>
         </is>
       </c>
-      <c r="D167" s="4" t="n">
-        <v>1487.16</v>
-      </c>
-      <c r="E167" s="4" t="n">
-        <v>174.944</v>
-      </c>
-      <c r="G167" s="4" t="n">
-        <v>18872.1</v>
+      <c r="D171" s="4" t="n">
+        <v>1490.08</v>
+      </c>
+      <c r="E171" s="4" t="n">
+        <v>174.963</v>
+      </c>
+      <c r="G171" s="4" t="n">
+        <v>19070.2</v>
+      </c>
+      <c r="I171" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J171" s="4" t="n">
+        <v>43.558</v>
+      </c>
+      <c r="K171" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -6465,7 +8157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6588,6 +8280,25 @@
       </c>
       <c r="E6" t="n">
         <v>7443</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="E7" t="n">
+        <v>198</v>
       </c>
     </row>
   </sheetData>
@@ -6633,13 +8344,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C2" t="n">
-        <v>1347.912</v>
+        <v>1350.832</v>
       </c>
       <c r="D2" t="n">
-        <v>161.643</v>
+        <v>161.662</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
update ha core and addons
</commit_message>
<xml_diff>
--- a/www/ev_charging_sessions.xlsx
+++ b/www/ev_charging_sessions.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sessions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Mesacny prehlad" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Pouzivatelia" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mesacny prehlad" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pouzivatelia" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K171"/>
+  <dimension ref="A1:K175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8122,27 +8122,207 @@
       </c>
     </row>
     <row r="171">
-      <c r="C171" s="4" t="inlineStr">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>01:29</t>
+        </is>
+      </c>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>mysan</t>
+        </is>
+      </c>
+      <c r="D171" s="3" t="n">
+        <v>8.259</v>
+      </c>
+      <c r="E171" s="3" t="n">
+        <v>0.998</v>
+      </c>
+      <c r="F171" s="2" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="G171" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="H171" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="I171" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J171" s="3" t="n">
+        <v>8.259</v>
+      </c>
+      <c r="K171" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>08:49</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>mysan</t>
+        </is>
+      </c>
+      <c r="D172" s="3" t="n">
+        <v>19.185</v>
+      </c>
+      <c r="E172" s="3" t="n">
+        <v>3.335</v>
+      </c>
+      <c r="F172" s="2" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G172" s="2" t="n">
+        <v>191.4</v>
+      </c>
+      <c r="H172" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="I172" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J172" s="3" t="n">
+        <v>19.185</v>
+      </c>
+      <c r="K172" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>14:46</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>mysan</t>
+        </is>
+      </c>
+      <c r="D173" s="3" t="n">
+        <v>18.685</v>
+      </c>
+      <c r="E173" s="3" t="n">
+        <v>2.451</v>
+      </c>
+      <c r="F173" s="2" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="G173" s="2" t="n">
+        <v>243.8</v>
+      </c>
+      <c r="H173" s="2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="I173" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J173" s="3" t="n">
+        <v>18.685</v>
+      </c>
+      <c r="K173" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>mysan</t>
+        </is>
+      </c>
+      <c r="D174" s="3" t="n">
+        <v>7.208</v>
+      </c>
+      <c r="E174" s="3" t="n">
+        <v>1.223</v>
+      </c>
+      <c r="F174" s="2" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="G174" s="2" t="n">
+        <v>135.7</v>
+      </c>
+      <c r="H174" s="2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="I174" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J174" s="3" t="n">
+        <v>7.208</v>
+      </c>
+      <c r="K174" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="C175" s="4" t="inlineStr">
         <is>
           <t>SPOLU:</t>
         </is>
       </c>
-      <c r="D171" s="4" t="n">
-        <v>1490.08</v>
-      </c>
-      <c r="E171" s="4" t="n">
-        <v>174.963</v>
-      </c>
-      <c r="G171" s="4" t="n">
-        <v>19070.2</v>
-      </c>
-      <c r="I171" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J171" s="4" t="n">
-        <v>43.558</v>
-      </c>
-      <c r="K171" s="4" t="n">
+      <c r="D175" s="4" t="n">
+        <v>1543.417</v>
+      </c>
+      <c r="E175" s="4" t="n">
+        <v>182.97</v>
+      </c>
+      <c r="G175" s="4" t="n">
+        <v>19720.1</v>
+      </c>
+      <c r="I175" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J175" s="4" t="n">
+        <v>96.895</v>
+      </c>
+      <c r="K175" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8289,16 +8469,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C7" t="n">
-        <v>2.92</v>
+        <v>56.257</v>
       </c>
       <c r="D7" t="n">
-        <v>0.019</v>
+        <v>8.026</v>
       </c>
       <c r="E7" t="n">
-        <v>198</v>
+        <v>848</v>
       </c>
     </row>
   </sheetData>
@@ -8344,13 +8524,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C2" t="n">
-        <v>1350.832</v>
+        <v>1404.169</v>
       </c>
       <c r="D2" t="n">
-        <v>161.662</v>
+        <v>169.669</v>
       </c>
     </row>
     <row r="3">

</xml_diff>